<commit_message>
db seed and clean up
</commit_message>
<xml_diff>
--- a/docs/SEED_DATA.xlsx
+++ b/docs/SEED_DATA.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="335">
   <si>
     <t>Section</t>
   </si>
@@ -80,10 +80,16 @@
     <t>make seed</t>
   </si>
   <si>
+    <t>Yopmail inbox</t>
+  </si>
+  <si>
+    <t>https://yopmail.com — enter the part before @yopmail.com (e.g. alice)</t>
+  </si>
+  <si>
     <t>Reset demo data</t>
   </si>
   <si>
-    <t>make seed (auto-cleans @demo.go-connect.local users first)</t>
+    <t>make seed (auto-cleans @yopmail.com users first)</t>
   </si>
   <si>
     <t>Name</t>
@@ -110,7 +116,7 @@
     <t>Demo Admin</t>
   </si>
   <si>
-    <t>admin@demo.go-connect.local</t>
+    <t>admin@yopmail.com</t>
   </si>
   <si>
     <t>admin</t>
@@ -125,7 +131,7 @@
     <t>Alice Sharma</t>
   </si>
   <si>
-    <t>alice@demo.go-connect.local</t>
+    <t>alice@yopmail.com</t>
   </si>
   <si>
     <t>customer</t>
@@ -137,7 +143,7 @@
     <t>Priya Patel</t>
   </si>
   <si>
-    <t>priya@demo.go-connect.local</t>
+    <t>priya@yopmail.com</t>
   </si>
   <si>
     <t>+919900010102</t>
@@ -146,7 +152,7 @@
     <t>Rahul Mehta</t>
   </si>
   <si>
-    <t>rahul@demo.go-connect.local</t>
+    <t>rahul@yopmail.com</t>
   </si>
   <si>
     <t>+919900010103</t>
@@ -155,7 +161,7 @@
     <t>Ananya Iyer</t>
   </si>
   <si>
-    <t>ananya@demo.go-connect.local</t>
+    <t>ananya@yopmail.com</t>
   </si>
   <si>
     <t>+919900010104</t>
@@ -164,7 +170,7 @@
     <t>Karim Hassan</t>
   </si>
   <si>
-    <t>karim@demo.go-connect.local</t>
+    <t>karim@yopmail.com</t>
   </si>
   <si>
     <t>employee</t>
@@ -176,7 +182,7 @@
     <t>Sara Khan</t>
   </si>
   <si>
-    <t>sara@demo.go-connect.local</t>
+    <t>sara@yopmail.com</t>
   </si>
   <si>
     <t>+919900020302</t>
@@ -185,7 +191,7 @@
     <t>Dev Reddy</t>
   </si>
   <si>
-    <t>dev@demo.go-connect.local</t>
+    <t>dev@yopmail.com</t>
   </si>
   <si>
     <t>+919900020303</t>
@@ -194,7 +200,7 @@
     <t>Meera Nair</t>
   </si>
   <si>
-    <t>meera@demo.go-connect.local</t>
+    <t>meera@yopmail.com</t>
   </si>
   <si>
     <t>+919900020304</t>
@@ -1336,87 +1342,87 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C3" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -1429,53 +1435,53 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -1488,53 +1494,53 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E1" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -1547,418 +1553,418 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D1" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E1" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="I2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E3" t="s">
+        <v>248</v>
+      </c>
+      <c r="F3" t="s">
+        <v>203</v>
+      </c>
+      <c r="G3" t="s">
+        <v>244</v>
+      </c>
+      <c r="H3" t="s">
         <v>245</v>
       </c>
-      <c r="B3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" t="s">
-        <v>132</v>
-      </c>
-      <c r="E3" t="s">
-        <v>246</v>
-      </c>
-      <c r="F3" t="s">
-        <v>201</v>
-      </c>
-      <c r="G3" t="s">
-        <v>242</v>
-      </c>
-      <c r="H3" t="s">
-        <v>243</v>
-      </c>
       <c r="I3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="J3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E4" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F4" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G4" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H4" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="I4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J4" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="G5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="H5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="I5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="F6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="G6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="I6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E7" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F7" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="G7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="H7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J7" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E8" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="H8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I8" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="J8" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E9" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F9" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G9" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="I9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J9" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E10" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="F10" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G10" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H10" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="I10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="J10" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D11" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E11" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G11" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="H11" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="I11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="J11" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D12" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E12" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G12" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="H12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I12" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J12" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F13" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G13" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H13" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="I13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J13" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -1971,117 +1977,117 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E1" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G1" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="F2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="F3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E4" t="s">
+        <v>298</v>
+      </c>
+      <c r="F4" t="s">
+        <v>96</v>
+      </c>
+      <c r="G4" t="s">
         <v>296</v>
-      </c>
-      <c r="F4" t="s">
-        <v>94</v>
-      </c>
-      <c r="G4" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E5" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="F5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G5" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -2094,121 +2100,121 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D1" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C4" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D4" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D5" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C6" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D6" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C7" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D7" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -2221,36 +2227,36 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C1" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D1" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E1" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="D2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E2" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -2263,36 +2269,36 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B1" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D1" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E1" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -2305,30 +2311,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B1" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C1" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -2411,6 +2417,14 @@
         <v>17</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -2421,45 +2435,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G2" t="s">
         <v>9</v>
@@ -2467,19 +2481,19 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
@@ -2490,19 +2504,19 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
         <v>10</v>
@@ -2513,19 +2527,19 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -2536,19 +2550,19 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
         <v>3</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
         <v>10</v>
@@ -2559,19 +2573,19 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F7" t="s">
         <v>12</v>
@@ -2582,19 +2596,19 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
         <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
         <v>12</v>
@@ -2605,19 +2619,19 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C9" t="s">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F9" t="s">
         <v>12</v>
@@ -2628,19 +2642,19 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F10" t="s">
         <v>12</v>
@@ -2659,128 +2673,128 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" t="s">
         <v>64</v>
-      </c>
-      <c r="C3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2793,177 +2807,177 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="J4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" t="s">
+        <v>119</v>
+      </c>
+      <c r="G5" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" t="s">
+        <v>121</v>
+      </c>
+      <c r="I5" t="s">
+        <v>122</v>
+      </c>
+      <c r="J5" t="s">
         <v>115</v>
       </c>
-      <c r="D5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="K5" t="s">
         <v>116</v>
-      </c>
-      <c r="F5" t="s">
-        <v>117</v>
-      </c>
-      <c r="G5" t="s">
-        <v>118</v>
-      </c>
-      <c r="H5" t="s">
-        <v>119</v>
-      </c>
-      <c r="I5" t="s">
-        <v>120</v>
-      </c>
-      <c r="J5" t="s">
-        <v>113</v>
-      </c>
-      <c r="K5" t="s">
-        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2976,236 +2990,236 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E5" t="s">
+        <v>145</v>
+      </c>
+      <c r="F5" t="s">
+        <v>146</v>
+      </c>
+      <c r="G5" t="s">
         <v>142</v>
       </c>
-      <c r="E5" t="s">
-        <v>143</v>
-      </c>
-      <c r="F5" t="s">
-        <v>144</v>
-      </c>
-      <c r="G5" t="s">
-        <v>140</v>
-      </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E8" t="s">
+        <v>158</v>
+      </c>
+      <c r="F8" t="s">
+        <v>159</v>
+      </c>
+      <c r="G8" t="s">
         <v>155</v>
       </c>
-      <c r="E8" t="s">
-        <v>156</v>
-      </c>
-      <c r="F8" t="s">
-        <v>157</v>
-      </c>
-      <c r="G8" t="s">
-        <v>153</v>
-      </c>
       <c r="H8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D9" t="s">
+        <v>162</v>
+      </c>
+      <c r="E9" t="s">
+        <v>163</v>
+      </c>
+      <c r="F9" t="s">
+        <v>164</v>
+      </c>
+      <c r="G9" t="s">
+        <v>132</v>
+      </c>
+      <c r="H9" t="s">
         <v>160</v>
-      </c>
-      <c r="E9" t="s">
-        <v>161</v>
-      </c>
-      <c r="F9" t="s">
-        <v>162</v>
-      </c>
-      <c r="G9" t="s">
-        <v>130</v>
-      </c>
-      <c r="H9" t="s">
-        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -3218,87 +3232,87 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -3311,163 +3325,163 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C3" t="s">
+        <v>188</v>
+      </c>
+      <c r="D3" t="s">
+        <v>184</v>
+      </c>
+      <c r="E3" t="s">
         <v>185</v>
       </c>
-      <c r="C3" t="s">
-        <v>186</v>
-      </c>
-      <c r="D3" t="s">
-        <v>182</v>
-      </c>
-      <c r="E3" t="s">
-        <v>183</v>
-      </c>
       <c r="F3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D4" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D6" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C7" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D7" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E7" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F7" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -3480,184 +3494,184 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C3" t="s">
         <v>203</v>
       </c>
-      <c r="C3" t="s">
-        <v>201</v>
-      </c>
       <c r="D3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
+        <v>206</v>
+      </c>
+      <c r="C4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D4" t="s">
         <v>204</v>
-      </c>
-      <c r="C4" t="s">
-        <v>201</v>
-      </c>
-      <c r="D4" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C5" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C7" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D7" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D8" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
+        <v>205</v>
+      </c>
+      <c r="C9" t="s">
         <v>203</v>
       </c>
-      <c r="C9" t="s">
-        <v>201</v>
-      </c>
       <c r="D9" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
+        <v>206</v>
+      </c>
+      <c r="C10" t="s">
+        <v>203</v>
+      </c>
+      <c r="D10" t="s">
         <v>204</v>
-      </c>
-      <c r="C10" t="s">
-        <v>201</v>
-      </c>
-      <c r="D10" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D11" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C12" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C13" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D13" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>